<commit_message>
5W-Programm KW30-34: Stellvertretung aus der Kopfzeile entfernt
Polier-Feld zeigt nur noch Samuel Decurtins.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/5W-Programm/Fuenfwochenprogramm_KW30-34.xlsx
+++ b/5W-Programm/Fuenfwochenprogramm_KW30-34.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stracloud-my.sharepoint.com/personal/maltvic_sbsit_com/Documents/Claude_Projects/Nalps_Ultra_KI/5W_Programm/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="11_391211456B66DE5FB370AC13A3B52B1DE327BE02" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AACE2A1-EDA6-440D-9980-5CA783270A42}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_391211456B66DE5FB370AC13A3B52B1DE327BE02" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{757CDE31-3BCF-4F9C-BC53-E9187C9FD7BC}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="720" yWindow="765" windowWidth="18945" windowHeight="9945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="223">
   <si>
     <t>5-Wochenprogramm</t>
   </si>
@@ -124,9 +124,6 @@
   </si>
   <si>
     <t>Polier</t>
-  </si>
-  <si>
-    <t>Samuel Decurtins (KW30 Ferien -&gt; Stv. Jorge)</t>
   </si>
   <si>
     <t>A --&gt; E = Anfang Ende Gesamtbauprogramm</t>
@@ -2909,7 +2906,7 @@
         <v>3</v>
       </c>
       <c r="P2" s="188" t="s">
-        <v>4</v>
+        <v>114</v>
       </c>
       <c r="Q2" s="174"/>
       <c r="R2" s="174"/>
@@ -2969,7 +2966,7 @@
     </row>
     <row r="3" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" s="186" t="str">
         <f>"Woche " &amp; WEEKNUM(B4)</f>
@@ -3059,7 +3056,7 @@
     </row>
     <row r="4" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="158">
         <f>B1</f>
@@ -3239,360 +3236,360 @@
     </row>
     <row r="5" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A5" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="181" t="s">
         <v>7</v>
-      </c>
-      <c r="B5" s="181" t="s">
-        <v>8</v>
       </c>
       <c r="C5" s="157"/>
       <c r="D5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E5" s="157"/>
       <c r="F5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" s="157"/>
       <c r="H5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I5" s="157"/>
       <c r="J5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K5" s="157"/>
       <c r="L5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M5" s="157"/>
       <c r="N5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O5" s="157"/>
       <c r="P5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q5" s="157"/>
       <c r="R5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S5" s="157"/>
       <c r="T5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U5" s="157"/>
       <c r="V5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="W5" s="157"/>
       <c r="X5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Y5" s="157"/>
       <c r="Z5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AA5" s="157"/>
       <c r="AB5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC5" s="157"/>
       <c r="AD5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AE5" s="157"/>
       <c r="AF5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AG5" s="157"/>
       <c r="AH5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AI5" s="157"/>
       <c r="AJ5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AK5" s="157"/>
       <c r="AL5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AM5" s="157"/>
       <c r="AN5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AO5" s="157"/>
       <c r="AP5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AQ5" s="157"/>
       <c r="AR5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AS5" s="157"/>
       <c r="AT5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AU5" s="157"/>
       <c r="AV5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AW5" s="157"/>
       <c r="AX5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AY5" s="157"/>
       <c r="AZ5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BA5" s="157"/>
       <c r="BB5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BC5" s="157"/>
       <c r="BD5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="BE5" s="157"/>
       <c r="BF5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="BG5" s="157"/>
       <c r="BH5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="BI5" s="157"/>
       <c r="BJ5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="BK5" s="157"/>
       <c r="BL5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="BM5" s="157"/>
       <c r="BN5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BO5" s="157"/>
       <c r="BP5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BQ5" s="157"/>
       <c r="BR5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="BS5" s="157"/>
     </row>
     <row r="6" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A6" s="14"/>
       <c r="B6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="F6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="H6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="J6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="L6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="N6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="P6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="R6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="T6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="U6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="U6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="V6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="X6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="Y6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Y6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="Z6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AA6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AA6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AB6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AC6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="AD6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AE6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AF6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AG6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AG6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AH6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AI6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AI6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AJ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AK6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AK6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AL6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AM6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AM6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AN6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AO6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AO6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AP6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AQ6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AQ6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="AR6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AS6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AS6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AT6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AU6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AU6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AV6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AW6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AW6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AX6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AY6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AY6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AZ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BA6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BA6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BB6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BC6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BC6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BD6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BE6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="BE6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="BF6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="BG6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BG6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BH6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BI6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BI6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BJ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BK6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BK6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BL6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BM6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BM6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BN6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BO6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BO6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BP6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BQ6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BQ6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BR6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BS6" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="BS6" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3743,7 +3740,7 @@
     </row>
     <row r="9" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A9" s="122" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" s="32"/>
       <c r="C9" s="31"/>
@@ -3818,7 +3815,7 @@
     </row>
     <row r="10" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A10" s="115" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" s="32"/>
       <c r="C10" s="31"/>
@@ -4039,7 +4036,7 @@
     </row>
     <row r="13" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A13" s="115" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="116"/>
       <c r="C13" s="117"/>
@@ -4114,7 +4111,7 @@
     </row>
     <row r="14" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A14" s="115" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="32"/>
       <c r="C14" s="31"/>
@@ -4262,7 +4259,7 @@
     </row>
     <row r="16" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A16" s="124" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B16" s="119"/>
       <c r="C16" s="120"/>
@@ -4337,7 +4334,7 @@
     </row>
     <row r="17" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A17" s="124" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="91"/>
       <c r="C17" s="92"/>
@@ -4412,7 +4409,7 @@
     </row>
     <row r="18" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A18" s="115" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" s="125"/>
       <c r="C18" s="31"/>
@@ -4487,7 +4484,7 @@
     </row>
     <row r="19" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A19" s="124" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B19" s="30"/>
       <c r="C19" s="31"/>
@@ -4562,7 +4559,7 @@
     </row>
     <row r="20" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A20" s="124" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B20" s="32"/>
       <c r="C20" s="31"/>
@@ -4637,7 +4634,7 @@
     </row>
     <row r="21" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A21" s="124" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" s="32"/>
       <c r="C21" s="31"/>
@@ -4712,7 +4709,7 @@
     </row>
     <row r="22" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A22" s="124" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B22" s="32"/>
       <c r="C22" s="31"/>
@@ -4787,7 +4784,7 @@
     </row>
     <row r="23" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A23" s="124" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23" s="94"/>
       <c r="C23" s="95"/>
@@ -4862,7 +4859,7 @@
     </row>
     <row r="24" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A24" s="124" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B24" s="32"/>
       <c r="C24" s="31"/>
@@ -4937,7 +4934,7 @@
     </row>
     <row r="25" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A25" s="124" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="31"/>
@@ -5012,7 +5009,7 @@
     </row>
     <row r="26" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A26" s="124" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B26" s="32"/>
       <c r="C26" s="31"/>
@@ -5087,7 +5084,7 @@
     </row>
     <row r="27" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A27" s="124" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27" s="32"/>
       <c r="C27" s="31"/>
@@ -5162,7 +5159,7 @@
     </row>
     <row r="28" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A28" s="124" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B28" s="32"/>
       <c r="C28" s="31"/>
@@ -5237,7 +5234,7 @@
     </row>
     <row r="29" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A29" s="115" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B29" s="32"/>
       <c r="C29" s="31"/>
@@ -5312,7 +5309,7 @@
     </row>
     <row r="30" spans="1:71" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="115" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B30" s="32"/>
       <c r="C30" s="31"/>
@@ -5460,7 +5457,7 @@
     </row>
     <row r="32" spans="1:71" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="122" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B32" s="32"/>
       <c r="C32" s="31"/>
@@ -5535,7 +5532,7 @@
     </row>
     <row r="33" spans="1:71" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="115" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B33" s="32"/>
       <c r="C33" s="31"/>
@@ -5610,7 +5607,7 @@
     </row>
     <row r="34" spans="1:71" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="115" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B34" s="32"/>
       <c r="C34" s="31"/>
@@ -5758,7 +5755,7 @@
     </row>
     <row r="36" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A36" s="126" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B36" s="32"/>
       <c r="C36" s="31"/>
@@ -5833,7 +5830,7 @@
     </row>
     <row r="37" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A37" s="127" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B37" s="32"/>
       <c r="C37" s="31"/>
@@ -5850,7 +5847,7 @@
       <c r="N37" s="26"/>
       <c r="O37" s="28"/>
       <c r="P37" s="128" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="Q37" s="31"/>
       <c r="R37" s="9"/>
@@ -5910,7 +5907,7 @@
     </row>
     <row r="38" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A38" s="129" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B38" s="32"/>
       <c r="C38" s="31"/>
@@ -5985,7 +5982,7 @@
     </row>
     <row r="39" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A39" s="129" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B39" s="49"/>
       <c r="C39" s="31"/>
@@ -6020,7 +6017,7 @@
       <c r="AF39" s="9"/>
       <c r="AG39" s="10"/>
       <c r="AH39" s="128" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AI39" s="10"/>
       <c r="AJ39" s="9"/>
@@ -6062,7 +6059,7 @@
     </row>
     <row r="40" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A40" s="129" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B40" s="128"/>
       <c r="C40" s="31"/>
@@ -6089,7 +6086,7 @@
       <c r="X40" s="54"/>
       <c r="Y40" s="10"/>
       <c r="Z40" s="134" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AA40" s="34"/>
       <c r="AB40" s="33"/>
@@ -6139,7 +6136,7 @@
     </row>
     <row r="41" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A41" s="129" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B41" s="128"/>
       <c r="C41" s="31"/>
@@ -6198,7 +6195,7 @@
       <c r="BD41" s="33"/>
       <c r="BE41" s="35"/>
       <c r="BF41" s="128" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="BG41" s="31"/>
       <c r="BH41" s="9"/>
@@ -6289,7 +6286,7 @@
     </row>
     <row r="43" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A43" s="130" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B43" s="49"/>
       <c r="C43" s="31"/>
@@ -6364,7 +6361,7 @@
     </row>
     <row r="44" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A44" s="129" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B44" s="100"/>
       <c r="C44" s="101"/>
@@ -6439,7 +6436,7 @@
     </row>
     <row r="45" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A45" s="127" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B45" s="32"/>
       <c r="C45" s="31"/>
@@ -6514,7 +6511,7 @@
     </row>
     <row r="46" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A46" s="127" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B46" s="32"/>
       <c r="C46" s="31"/>
@@ -6589,7 +6586,7 @@
     </row>
     <row r="47" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A47" s="127" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B47" s="32"/>
       <c r="C47" s="31"/>
@@ -6664,7 +6661,7 @@
     </row>
     <row r="48" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A48" s="127" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B48" s="32"/>
       <c r="C48" s="31"/>
@@ -6739,7 +6736,7 @@
     </row>
     <row r="49" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A49" s="127" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B49" s="32"/>
       <c r="C49" s="31"/>
@@ -6814,7 +6811,7 @@
     </row>
     <row r="50" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A50" s="127" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B50" s="32"/>
       <c r="C50" s="31"/>
@@ -6889,7 +6886,7 @@
     </row>
     <row r="51" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A51" s="127" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B51" s="32"/>
       <c r="C51" s="31"/>
@@ -6964,7 +6961,7 @@
     </row>
     <row r="52" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A52" s="127" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B52" s="32"/>
       <c r="C52" s="31"/>
@@ -7039,7 +7036,7 @@
     </row>
     <row r="53" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A53" s="127" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B53" s="32"/>
       <c r="C53" s="31"/>
@@ -7114,7 +7111,7 @@
     </row>
     <row r="54" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A54" s="127" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B54" s="32"/>
       <c r="C54" s="31"/>
@@ -7189,7 +7186,7 @@
     </row>
     <row r="55" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A55" s="127" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B55" s="32"/>
       <c r="C55" s="31"/>
@@ -7264,7 +7261,7 @@
     </row>
     <row r="56" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A56" s="126" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B56" s="32"/>
       <c r="C56" s="31"/>
@@ -7339,7 +7336,7 @@
     </row>
     <row r="57" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A57" s="127" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B57" s="103"/>
       <c r="C57" s="104"/>
@@ -7414,7 +7411,7 @@
     </row>
     <row r="58" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A58" s="127" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B58" s="32"/>
       <c r="C58" s="31"/>
@@ -7489,7 +7486,7 @@
     </row>
     <row r="59" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A59" s="127" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B59" s="32"/>
       <c r="C59" s="31"/>
@@ -7564,7 +7561,7 @@
     </row>
     <row r="60" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A60" s="127" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B60" s="32"/>
       <c r="C60" s="31"/>
@@ -7712,7 +7709,7 @@
     </row>
     <row r="62" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A62" s="126" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B62" s="32"/>
       <c r="C62" s="31"/>
@@ -7787,7 +7784,7 @@
     </row>
     <row r="63" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A63" s="127" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B63" s="32"/>
       <c r="C63" s="31"/>
@@ -7862,7 +7859,7 @@
     </row>
     <row r="64" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A64" s="127" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B64" s="32"/>
       <c r="C64" s="31"/>
@@ -7937,7 +7934,7 @@
     </row>
     <row r="65" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A65" s="127" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B65" s="32"/>
       <c r="C65" s="31"/>
@@ -8158,7 +8155,7 @@
     </row>
     <row r="68" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A68" s="126" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B68" s="32"/>
       <c r="C68" s="31"/>
@@ -8233,7 +8230,7 @@
     </row>
     <row r="69" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A69" s="127" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B69" s="109"/>
       <c r="C69" s="110"/>
@@ -8308,7 +8305,7 @@
     </row>
     <row r="70" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A70" s="127" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B70" s="119"/>
       <c r="C70" s="120"/>
@@ -8383,7 +8380,7 @@
     </row>
     <row r="71" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A71" s="127" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B71" s="32"/>
       <c r="C71" s="31"/>
@@ -8458,7 +8455,7 @@
     </row>
     <row r="72" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A72" s="127" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B72" s="109"/>
       <c r="C72" s="110"/>
@@ -8533,7 +8530,7 @@
     </row>
     <row r="73" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A73" s="127" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B73" s="32"/>
       <c r="C73" s="31"/>
@@ -8608,7 +8605,7 @@
     </row>
     <row r="74" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A74" s="127" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B74" s="32"/>
       <c r="C74" s="31"/>
@@ -8683,7 +8680,7 @@
     </row>
     <row r="75" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A75" s="127" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B75" s="32"/>
       <c r="C75" s="31"/>
@@ -8758,7 +8755,7 @@
     </row>
     <row r="76" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A76" s="131" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B76" s="32"/>
       <c r="C76" s="31"/>
@@ -8833,7 +8830,7 @@
     </row>
     <row r="77" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A77" s="115" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B77" s="32"/>
       <c r="C77" s="31"/>
@@ -8908,7 +8905,7 @@
     </row>
     <row r="78" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A78" s="115" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B78" s="32"/>
       <c r="C78" s="31"/>
@@ -8983,7 +8980,7 @@
     </row>
     <row r="79" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A79" s="115" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B79" s="112"/>
       <c r="C79" s="113"/>
@@ -9058,7 +9055,7 @@
     </row>
     <row r="80" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A80" s="115" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B80" s="32"/>
       <c r="C80" s="31"/>
@@ -9133,7 +9130,7 @@
     </row>
     <row r="81" spans="1:71" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="131" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B81" s="32"/>
       <c r="C81" s="31"/>
@@ -9164,7 +9161,7 @@
       <c r="AB81" s="33"/>
       <c r="AC81" s="35"/>
       <c r="AD81" s="128" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AE81" s="31"/>
       <c r="AF81" s="9"/>
@@ -9210,7 +9207,7 @@
     </row>
     <row r="82" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A82" s="131" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B82" s="32"/>
       <c r="C82" s="31"/>
@@ -9233,7 +9230,7 @@
       <c r="T82" s="9"/>
       <c r="U82" s="10"/>
       <c r="V82" s="132" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="W82" s="10"/>
       <c r="X82" s="9"/>
@@ -9287,7 +9284,7 @@
     </row>
     <row r="83" spans="1:71" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="131" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B83" s="109"/>
       <c r="C83" s="110"/>
@@ -9362,7 +9359,7 @@
     </row>
     <row r="84" spans="1:71" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="131" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B84" s="32"/>
       <c r="C84" s="31"/>
@@ -9437,7 +9434,7 @@
     </row>
     <row r="85" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A85" s="131" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B85" s="32"/>
       <c r="C85" s="31"/>
@@ -9512,7 +9509,7 @@
     </row>
     <row r="86" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A86" s="131" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B86" s="32"/>
       <c r="C86" s="31"/>
@@ -9660,7 +9657,7 @@
     </row>
     <row r="88" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A88" s="126" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B88" s="32"/>
       <c r="C88" s="31"/>
@@ -9735,7 +9732,7 @@
     </row>
     <row r="89" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A89" s="127" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B89" s="112"/>
       <c r="C89" s="113"/>
@@ -9810,7 +9807,7 @@
     </row>
     <row r="90" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A90" s="127" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B90" s="112"/>
       <c r="C90" s="113"/>
@@ -9885,7 +9882,7 @@
     </row>
     <row r="91" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A91" s="127" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B91" s="112"/>
       <c r="C91" s="113"/>
@@ -9960,7 +9957,7 @@
     </row>
     <row r="92" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A92" s="127" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B92" s="32"/>
       <c r="C92" s="113"/>
@@ -10035,7 +10032,7 @@
     </row>
     <row r="93" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A93" s="127" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B93" s="32"/>
       <c r="C93" s="31"/>
@@ -10110,7 +10107,7 @@
     </row>
     <row r="94" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A94" s="127" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B94" s="32"/>
       <c r="C94" s="31"/>
@@ -10185,7 +10182,7 @@
     </row>
     <row r="95" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A95" s="126" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B95" s="32"/>
       <c r="C95" s="31"/>
@@ -10260,7 +10257,7 @@
     </row>
     <row r="96" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A96" s="126" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B96" s="32"/>
       <c r="C96" s="31"/>
@@ -10335,10 +10332,10 @@
     </row>
     <row r="97" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A97" s="127" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B97" s="128" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C97" s="31"/>
       <c r="D97" s="9"/>
@@ -10412,7 +10409,7 @@
     </row>
     <row r="98" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A98" s="127" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B98" s="32"/>
       <c r="C98" s="31"/>
@@ -10487,7 +10484,7 @@
     </row>
     <row r="99" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A99" s="127" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B99" s="32"/>
       <c r="C99" s="31"/>
@@ -10510,7 +10507,7 @@
       <c r="T99" s="9"/>
       <c r="U99" s="10"/>
       <c r="V99" s="132" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="W99" s="10"/>
       <c r="X99" s="9"/>
@@ -10564,7 +10561,7 @@
     </row>
     <row r="100" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A100" s="127" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B100" s="32"/>
       <c r="C100" s="31"/>
@@ -10639,7 +10636,7 @@
     </row>
     <row r="101" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A101" s="127" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B101" s="32"/>
       <c r="C101" s="31"/>
@@ -10714,7 +10711,7 @@
     </row>
     <row r="102" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A102" s="127" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B102" s="32"/>
       <c r="C102" s="31"/>
@@ -10789,7 +10786,7 @@
     </row>
     <row r="103" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A103" s="127" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B103" s="32"/>
       <c r="C103" s="31"/>
@@ -10822,7 +10819,7 @@
       <c r="AD103" s="32"/>
       <c r="AE103" s="31"/>
       <c r="AF103" s="132" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AG103" s="10"/>
       <c r="AH103" s="9"/>
@@ -10866,10 +10863,10 @@
     </row>
     <row r="104" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A104" s="127" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B104" s="128" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C104" s="31"/>
       <c r="D104" s="9"/>
@@ -10943,7 +10940,7 @@
     </row>
     <row r="105" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A105" s="129" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B105" s="32"/>
       <c r="C105" s="31"/>
@@ -11018,7 +11015,7 @@
     </row>
     <row r="106" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A106" s="129" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B106" s="32"/>
       <c r="C106" s="31"/>
@@ -11093,7 +11090,7 @@
     </row>
     <row r="107" spans="1:71" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A107" s="129" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B107" s="32"/>
       <c r="C107" s="31"/>
@@ -11168,7 +11165,7 @@
     </row>
     <row r="108" spans="1:71" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A108" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B108" s="176">
         <v>22</v>
@@ -11313,7 +11310,7 @@
     </row>
     <row r="109" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B109" s="153"/>
       <c r="C109" s="154"/>
@@ -11389,7 +11386,7 @@
     <row r="110" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="177"/>
       <c r="B110" s="162" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C110" s="163"/>
       <c r="D110" s="163"/>
@@ -11405,7 +11402,7 @@
       <c r="N110" s="163"/>
       <c r="O110" s="164"/>
       <c r="P110" s="162" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="Q110" s="163"/>
       <c r="R110" s="163"/>
@@ -11421,7 +11418,7 @@
       <c r="AB110" s="163"/>
       <c r="AC110" s="164"/>
       <c r="AD110" s="162" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="AE110" s="163"/>
       <c r="AF110" s="163"/>
@@ -11437,7 +11434,7 @@
       <c r="AP110" s="163"/>
       <c r="AQ110" s="164"/>
       <c r="AR110" s="162" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AS110" s="163"/>
       <c r="AT110" s="163"/>
@@ -11453,7 +11450,7 @@
       <c r="BD110" s="163"/>
       <c r="BE110" s="164"/>
       <c r="BF110" s="162" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="BG110" s="163"/>
       <c r="BH110" s="163"/>
@@ -12158,7 +12155,7 @@
         <v>3</v>
       </c>
       <c r="P2" s="188" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="Q2" s="174"/>
       <c r="R2" s="174"/>
@@ -12218,7 +12215,7 @@
     </row>
     <row r="3" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" s="186" t="str">
         <f>"Woche " &amp; WEEKNUM(B4)</f>
@@ -12308,7 +12305,7 @@
     </row>
     <row r="4" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="158">
         <f>B1</f>
@@ -12488,360 +12485,360 @@
     </row>
     <row r="5" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A5" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="181" t="s">
         <v>7</v>
-      </c>
-      <c r="B5" s="181" t="s">
-        <v>8</v>
       </c>
       <c r="C5" s="157"/>
       <c r="D5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E5" s="157"/>
       <c r="F5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" s="157"/>
       <c r="H5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I5" s="157"/>
       <c r="J5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K5" s="157"/>
       <c r="L5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M5" s="157"/>
       <c r="N5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O5" s="157"/>
       <c r="P5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q5" s="157"/>
       <c r="R5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S5" s="157"/>
       <c r="T5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U5" s="157"/>
       <c r="V5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="W5" s="157"/>
       <c r="X5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Y5" s="157"/>
       <c r="Z5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AA5" s="157"/>
       <c r="AB5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC5" s="157"/>
       <c r="AD5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AE5" s="157"/>
       <c r="AF5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AG5" s="157"/>
       <c r="AH5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AI5" s="157"/>
       <c r="AJ5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AK5" s="157"/>
       <c r="AL5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AM5" s="157"/>
       <c r="AN5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AO5" s="157"/>
       <c r="AP5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AQ5" s="157"/>
       <c r="AR5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AS5" s="157"/>
       <c r="AT5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AU5" s="157"/>
       <c r="AV5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AW5" s="157"/>
       <c r="AX5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AY5" s="157"/>
       <c r="AZ5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BA5" s="157"/>
       <c r="BB5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BC5" s="157"/>
       <c r="BD5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="BE5" s="157"/>
       <c r="BF5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="BG5" s="157"/>
       <c r="BH5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="BI5" s="157"/>
       <c r="BJ5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="BK5" s="157"/>
       <c r="BL5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="BM5" s="157"/>
       <c r="BN5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BO5" s="157"/>
       <c r="BP5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BQ5" s="157"/>
       <c r="BR5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="BS5" s="157"/>
     </row>
     <row r="6" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A6" s="14"/>
       <c r="B6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="F6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="H6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="J6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="L6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="N6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="P6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="R6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="T6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="U6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="U6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="V6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="X6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="Y6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Y6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="Z6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AA6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AA6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AB6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AC6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="AD6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AE6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AF6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AG6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AG6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AH6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AI6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AI6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AJ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AK6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AK6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AL6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AM6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AM6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AN6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AO6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AO6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AP6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AQ6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AQ6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="AR6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AS6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AS6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AT6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AU6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AU6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AV6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AW6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AW6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AX6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AY6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AY6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AZ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BA6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BA6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BB6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BC6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BC6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BD6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BE6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="BE6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="BF6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="BG6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BG6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BH6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BI6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BI6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BJ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BK6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BK6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BL6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BM6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BM6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BN6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BO6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BO6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BP6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BQ6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BQ6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BR6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BS6" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="BS6" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -12919,7 +12916,7 @@
     </row>
     <row r="8" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="65" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B8" s="32"/>
       <c r="C8" s="31"/>
@@ -12994,7 +12991,7 @@
     </row>
     <row r="9" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="69" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B9" s="43"/>
       <c r="C9" s="44"/>
@@ -13653,7 +13650,7 @@
     </row>
     <row r="18" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A18" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="31"/>
@@ -13728,7 +13725,7 @@
     </row>
     <row r="19" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A19" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B19" s="32"/>
       <c r="C19" s="31"/>
@@ -13803,7 +13800,7 @@
     </row>
     <row r="20" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A20" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B20" s="32"/>
       <c r="C20" s="31"/>
@@ -13878,7 +13875,7 @@
     </row>
     <row r="21" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B21" s="32"/>
       <c r="C21" s="31"/>
@@ -13953,7 +13950,7 @@
     </row>
     <row r="22" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A22" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B22" s="32"/>
       <c r="C22" s="31"/>
@@ -14028,7 +14025,7 @@
     </row>
     <row r="23" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A23" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B23" s="32"/>
       <c r="C23" s="31"/>
@@ -14047,7 +14044,7 @@
       <c r="P23" s="48"/>
       <c r="Q23" s="47"/>
       <c r="R23" s="77" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="S23" s="55"/>
       <c r="T23" s="46"/>
@@ -14105,7 +14102,7 @@
     </row>
     <row r="24" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A24" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B24" s="32"/>
       <c r="C24" s="31"/>
@@ -14180,7 +14177,7 @@
     </row>
     <row r="25" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A25" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="31"/>
@@ -14255,7 +14252,7 @@
     </row>
     <row r="26" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A26" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B26" s="32"/>
       <c r="C26" s="31"/>
@@ -14330,7 +14327,7 @@
     </row>
     <row r="27" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A27" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B27" s="32"/>
       <c r="C27" s="31"/>
@@ -14478,7 +14475,7 @@
     </row>
     <row r="29" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A29" s="18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B29" s="32"/>
       <c r="C29" s="31"/>
@@ -14553,7 +14550,7 @@
     </row>
     <row r="30" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A30" s="36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B30" s="32"/>
       <c r="C30" s="31"/>
@@ -14628,7 +14625,7 @@
     </row>
     <row r="31" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A31" s="53" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B31" s="32"/>
       <c r="C31" s="31"/>
@@ -14703,7 +14700,7 @@
     </row>
     <row r="32" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A32" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B32" s="72"/>
       <c r="C32" s="20"/>
@@ -14726,7 +14723,7 @@
       <c r="T32" s="46"/>
       <c r="U32" s="47"/>
       <c r="V32" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="W32" s="10"/>
       <c r="X32" s="9"/>
@@ -14739,7 +14736,7 @@
       <c r="AE32" s="31"/>
       <c r="AF32" s="9"/>
       <c r="AG32" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AH32" s="9"/>
       <c r="AI32" s="10"/>
@@ -14782,17 +14779,17 @@
     </row>
     <row r="33" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A33" s="71" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="9"/>
       <c r="E33" s="10"/>
       <c r="F33" s="29"/>
       <c r="G33" s="20" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H33" s="29"/>
       <c r="I33" s="20"/>
@@ -14861,7 +14858,7 @@
     </row>
     <row r="34" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A34" s="71" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B34" s="32"/>
       <c r="C34" s="31"/>
@@ -14870,7 +14867,7 @@
       <c r="F34" s="9"/>
       <c r="G34" s="10"/>
       <c r="H34" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I34" s="10"/>
       <c r="J34" s="29"/>
@@ -14885,7 +14882,7 @@
       <c r="S34" s="20"/>
       <c r="T34" s="29"/>
       <c r="U34" s="20" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="V34" s="29"/>
       <c r="W34" s="10"/>
@@ -14940,7 +14937,7 @@
     </row>
     <row r="35" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A35" s="36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B35" s="32"/>
       <c r="C35" s="31"/>
@@ -14975,10 +14972,10 @@
       <c r="AF35" s="9"/>
       <c r="AG35" s="10"/>
       <c r="AH35" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="AI35" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="AI35" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="AJ35" s="46"/>
       <c r="AK35" s="47"/>
@@ -15019,7 +15016,7 @@
     </row>
     <row r="36" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A36" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B36" s="32"/>
       <c r="C36" s="31"/>
@@ -15058,7 +15055,7 @@
       <c r="AJ36" s="46"/>
       <c r="AK36" s="47"/>
       <c r="AL36" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AM36" s="10"/>
       <c r="AN36" s="26"/>
@@ -15067,7 +15064,7 @@
       <c r="AQ36" s="28"/>
       <c r="AR36" s="32"/>
       <c r="AS36" s="31" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AT36" s="9"/>
       <c r="AU36" s="10"/>
@@ -15098,7 +15095,7 @@
     </row>
     <row r="37" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A37" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B37" s="32"/>
       <c r="C37" s="31"/>
@@ -15145,10 +15142,10 @@
       <c r="AR37" s="32"/>
       <c r="AS37" s="31"/>
       <c r="AT37" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU37" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="AU37" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="AV37" s="9"/>
       <c r="AW37" s="10"/>
@@ -15177,7 +15174,7 @@
     </row>
     <row r="38" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A38" s="36" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B38" s="32"/>
       <c r="C38" s="31"/>
@@ -15226,7 +15223,7 @@
       <c r="AT38" s="9"/>
       <c r="AU38" s="10"/>
       <c r="AV38" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AW38" s="10"/>
       <c r="AX38" s="9"/>
@@ -15239,7 +15236,7 @@
       <c r="BE38" s="28"/>
       <c r="BF38" s="32"/>
       <c r="BG38" s="31" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="BH38" s="9"/>
       <c r="BI38" s="10"/>
@@ -15256,7 +15253,7 @@
     </row>
     <row r="39" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A39" s="36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B39" s="32"/>
       <c r="C39" s="31"/>
@@ -15317,14 +15314,14 @@
       <c r="BF39" s="32"/>
       <c r="BG39" s="31"/>
       <c r="BH39" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="BI39" s="10"/>
       <c r="BJ39" s="9"/>
       <c r="BK39" s="10"/>
       <c r="BL39" s="9"/>
       <c r="BM39" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="BN39" s="9"/>
       <c r="BO39" s="10"/>
@@ -15408,7 +15405,7 @@
     </row>
     <row r="41" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A41" s="36" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B41" s="32"/>
       <c r="C41" s="31"/>
@@ -15441,10 +15438,10 @@
       <c r="AD41" s="32"/>
       <c r="AE41" s="31"/>
       <c r="AF41" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="AG41" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="AG41" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="AH41" s="9"/>
       <c r="AI41" s="10"/>
@@ -15487,7 +15484,7 @@
     </row>
     <row r="42" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A42" s="36" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B42" s="32"/>
       <c r="C42" s="31"/>
@@ -15552,10 +15549,10 @@
       <c r="BJ42" s="9"/>
       <c r="BK42" s="10"/>
       <c r="BL42" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="BM42" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="BM42" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="BN42" s="9"/>
       <c r="BO42" s="10"/>
@@ -16077,7 +16074,7 @@
     </row>
     <row r="50" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A50" s="65" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B50" s="32"/>
       <c r="C50" s="31"/>
@@ -16152,7 +16149,7 @@
     </row>
     <row r="51" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A51" s="65" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B51" s="32"/>
       <c r="C51" s="31"/>
@@ -16227,7 +16224,7 @@
     </row>
     <row r="52" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A52" s="67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B52" s="32"/>
       <c r="C52" s="31"/>
@@ -16302,14 +16299,14 @@
     </row>
     <row r="53" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A53" s="67" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B53" s="49"/>
       <c r="C53" s="31"/>
       <c r="D53" s="9"/>
       <c r="E53" s="10"/>
       <c r="F53" s="54" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G53" s="10"/>
       <c r="H53" s="9"/>
@@ -16379,7 +16376,7 @@
     </row>
     <row r="54" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A54" s="67" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B54" s="49"/>
       <c r="C54" s="31"/>
@@ -16410,7 +16407,7 @@
       <c r="AB54" s="33"/>
       <c r="AC54" s="35"/>
       <c r="AD54" s="49" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AE54" s="31"/>
       <c r="AF54" s="9"/>
@@ -16456,7 +16453,7 @@
     </row>
     <row r="55" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A55" s="67" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B55" s="49"/>
       <c r="C55" s="31"/>
@@ -16750,7 +16747,7 @@
     </row>
     <row r="59" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A59" s="65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B59" s="32"/>
       <c r="C59" s="31"/>
@@ -16825,7 +16822,7 @@
     </row>
     <row r="60" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A60" s="66" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B60" s="70"/>
       <c r="C60" s="55"/>
@@ -16900,7 +16897,7 @@
     </row>
     <row r="61" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A61" s="66" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B61" s="32"/>
       <c r="C61" s="31"/>
@@ -16975,7 +16972,7 @@
     </row>
     <row r="62" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A62" s="66" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B62" s="32"/>
       <c r="C62" s="10"/>
@@ -17050,7 +17047,7 @@
     </row>
     <row r="63" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A63" s="66" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B63" s="32"/>
       <c r="C63" s="31"/>
@@ -17271,7 +17268,7 @@
     </row>
     <row r="66" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A66" s="65" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B66" s="32"/>
       <c r="C66" s="31"/>
@@ -17346,7 +17343,7 @@
     </row>
     <row r="67" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A67" s="65" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B67" s="32"/>
       <c r="C67" s="31"/>
@@ -17421,7 +17418,7 @@
     </row>
     <row r="68" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A68" s="66" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B68" s="32"/>
       <c r="C68" s="31"/>
@@ -17445,11 +17442,11 @@
       <c r="U68" s="47"/>
       <c r="V68" s="10"/>
       <c r="W68" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="X68" s="9"/>
       <c r="Y68" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Z68" s="33"/>
       <c r="AA68" s="34"/>
@@ -17500,7 +17497,7 @@
     </row>
     <row r="69" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A69" s="66" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B69" s="32"/>
       <c r="C69" s="31"/>
@@ -17519,7 +17516,7 @@
       <c r="P69" s="48"/>
       <c r="Q69" s="47"/>
       <c r="R69" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="S69" s="10"/>
       <c r="T69" s="46"/>
@@ -17542,7 +17539,7 @@
       <c r="AK69" s="47"/>
       <c r="AL69" s="9"/>
       <c r="AM69" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AN69" s="33"/>
       <c r="AO69" s="34"/>
@@ -17579,7 +17576,7 @@
     </row>
     <row r="70" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A70" s="66" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B70" s="32"/>
       <c r="C70" s="31"/>
@@ -17624,7 +17621,7 @@
       <c r="AP70" s="33"/>
       <c r="AQ70" s="35"/>
       <c r="AR70" s="32" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AS70" s="31"/>
       <c r="AT70" s="9"/>
@@ -17643,7 +17640,7 @@
       <c r="BG70" s="31"/>
       <c r="BH70" s="9"/>
       <c r="BI70" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="BJ70" s="9"/>
       <c r="BK70" s="10"/>
@@ -17658,7 +17655,7 @@
     </row>
     <row r="71" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A71" s="66" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B71" s="32"/>
       <c r="C71" s="31"/>
@@ -17721,7 +17718,7 @@
       <c r="BH71" s="9"/>
       <c r="BI71" s="10"/>
       <c r="BJ71" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="BK71" s="10"/>
       <c r="BL71" s="9"/>
@@ -17735,7 +17732,7 @@
     </row>
     <row r="72" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A72" s="66" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B72" s="32"/>
       <c r="C72" s="31"/>
@@ -17794,14 +17791,14 @@
       <c r="BD72" s="33"/>
       <c r="BE72" s="35"/>
       <c r="BF72" s="32" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="BG72" s="31"/>
       <c r="BH72" s="9"/>
       <c r="BI72" s="10"/>
       <c r="BJ72" s="9"/>
       <c r="BK72" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="BL72" s="9"/>
       <c r="BM72" s="10"/>
@@ -17887,7 +17884,7 @@
     </row>
     <row r="74" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A74" s="66" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B74" s="32"/>
       <c r="C74" s="31"/>
@@ -17962,7 +17959,7 @@
     </row>
     <row r="75" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A75" s="66" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B75" s="32"/>
       <c r="C75" s="31"/>
@@ -18037,7 +18034,7 @@
     </row>
     <row r="76" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A76" s="66" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B76" s="32"/>
       <c r="C76" s="31"/>
@@ -18185,7 +18182,7 @@
     </row>
     <row r="78" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A78" s="66" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B78" s="32"/>
       <c r="C78" s="31"/>
@@ -18406,7 +18403,7 @@
     </row>
     <row r="81" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A81" s="65" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B81" s="32"/>
       <c r="C81" s="31"/>
@@ -18481,7 +18478,7 @@
     </row>
     <row r="82" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A82" s="66" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B82" s="32"/>
       <c r="C82" s="31"/>
@@ -18556,7 +18553,7 @@
     </row>
     <row r="83" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A83" s="66" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B83" s="32"/>
       <c r="C83" s="31"/>
@@ -18631,7 +18628,7 @@
     </row>
     <row r="84" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A84" s="66" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B84" s="32"/>
       <c r="C84" s="31"/>
@@ -18706,7 +18703,7 @@
     </row>
     <row r="85" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A85" s="66" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B85" s="32"/>
       <c r="C85" s="31"/>
@@ -18781,7 +18778,7 @@
     </row>
     <row r="86" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A86" s="66" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B86" s="32"/>
       <c r="C86" s="31"/>
@@ -18856,7 +18853,7 @@
     </row>
     <row r="87" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A87" s="66" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B87" s="32"/>
       <c r="C87" s="31"/>
@@ -18931,7 +18928,7 @@
     </row>
     <row r="88" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A88" s="66" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B88" s="32"/>
       <c r="C88" s="31"/>
@@ -19006,7 +19003,7 @@
     </row>
     <row r="89" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A89" s="66" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B89" s="32"/>
       <c r="C89" s="31"/>
@@ -19154,7 +19151,7 @@
     </row>
     <row r="91" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A91" s="18" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B91" s="32"/>
       <c r="C91" s="31"/>
@@ -19229,7 +19226,7 @@
     </row>
     <row r="92" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A92" s="15" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B92" s="41"/>
       <c r="C92" s="42"/>
@@ -19304,7 +19301,7 @@
     </row>
     <row r="93" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A93" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B93" s="59"/>
       <c r="C93" s="10"/>
@@ -19379,7 +19376,7 @@
     </row>
     <row r="94" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A94" s="15" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B94" s="32"/>
       <c r="C94" s="31"/>
@@ -19454,7 +19451,7 @@
     </row>
     <row r="95" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A95" s="45" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B95" s="59"/>
       <c r="C95" s="10"/>
@@ -19529,7 +19526,7 @@
     </row>
     <row r="96" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A96" s="45" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B96" s="32"/>
       <c r="C96" s="31"/>
@@ -19604,7 +19601,7 @@
     </row>
     <row r="97" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A97" s="45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B97" s="32"/>
       <c r="C97" s="31"/>
@@ -19679,7 +19676,7 @@
     </row>
     <row r="98" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A98" s="45" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B98" s="32"/>
       <c r="C98" s="31"/>
@@ -19754,7 +19751,7 @@
     </row>
     <row r="99" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A99" s="45" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B99" s="32"/>
       <c r="C99" s="31"/>
@@ -19974,7 +19971,7 @@
     </row>
     <row r="102" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A102" s="65" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B102" s="32"/>
       <c r="C102" s="31"/>
@@ -20049,7 +20046,7 @@
     </row>
     <row r="103" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A103" s="65" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B103" s="32"/>
       <c r="C103" s="31"/>
@@ -20270,7 +20267,7 @@
     </row>
     <row r="106" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A106" s="65" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B106" s="32"/>
       <c r="C106" s="31"/>
@@ -20345,7 +20342,7 @@
     </row>
     <row r="107" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A107" s="66" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B107" s="32"/>
       <c r="C107" s="31"/>
@@ -20493,7 +20490,7 @@
     </row>
     <row r="109" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A109" s="65" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B109" s="32"/>
       <c r="C109" s="31"/>
@@ -20568,7 +20565,7 @@
     </row>
     <row r="110" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A110" s="66" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B110" s="32"/>
       <c r="C110" s="31"/>
@@ -20643,7 +20640,7 @@
     </row>
     <row r="111" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A111" s="66" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B111" s="32"/>
       <c r="C111" s="31"/>
@@ -20718,7 +20715,7 @@
     </row>
     <row r="112" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A112" s="66" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B112" s="32"/>
       <c r="C112" s="31"/>
@@ -20866,7 +20863,7 @@
     </row>
     <row r="114" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A114" s="65" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B114" s="32"/>
       <c r="C114" s="31"/>
@@ -21452,7 +21449,7 @@
     </row>
     <row r="122" spans="1:71" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A122" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B122" s="176">
         <v>22</v>
@@ -21597,7 +21594,7 @@
     </row>
     <row r="123" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B123" s="153"/>
       <c r="C123" s="154"/>
@@ -21673,7 +21670,7 @@
     <row r="124" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="177"/>
       <c r="B124" s="191" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C124" s="163"/>
       <c r="D124" s="163"/>
@@ -21689,7 +21686,7 @@
       <c r="N124" s="163"/>
       <c r="O124" s="164"/>
       <c r="P124" s="191" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q124" s="163"/>
       <c r="R124" s="163"/>
@@ -21719,7 +21716,7 @@
       <c r="AP124" s="163"/>
       <c r="AQ124" s="164"/>
       <c r="AR124" s="191" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AS124" s="163"/>
       <c r="AT124" s="163"/>
@@ -21735,7 +21732,7 @@
       <c r="BD124" s="163"/>
       <c r="BE124" s="164"/>
       <c r="BF124" s="191" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="BG124" s="163"/>
       <c r="BH124" s="163"/>
@@ -22441,7 +22438,7 @@
         <v>3</v>
       </c>
       <c r="P2" s="188" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="Q2" s="174"/>
       <c r="R2" s="174"/>
@@ -22768,357 +22765,357 @@
     <row r="5" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A5" s="75"/>
       <c r="B5" s="181" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" s="157"/>
       <c r="D5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E5" s="157"/>
       <c r="F5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" s="157"/>
       <c r="H5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I5" s="157"/>
       <c r="J5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K5" s="157"/>
       <c r="L5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M5" s="157"/>
       <c r="N5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O5" s="157"/>
       <c r="P5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q5" s="157"/>
       <c r="R5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S5" s="157"/>
       <c r="T5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U5" s="157"/>
       <c r="V5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="W5" s="157"/>
       <c r="X5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Y5" s="157"/>
       <c r="Z5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AA5" s="157"/>
       <c r="AB5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC5" s="157"/>
       <c r="AD5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AE5" s="157"/>
       <c r="AF5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AG5" s="157"/>
       <c r="AH5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AI5" s="157"/>
       <c r="AJ5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AK5" s="157"/>
       <c r="AL5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AM5" s="157"/>
       <c r="AN5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AO5" s="157"/>
       <c r="AP5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AQ5" s="157"/>
       <c r="AR5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AS5" s="157"/>
       <c r="AT5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AU5" s="157"/>
       <c r="AV5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AW5" s="157"/>
       <c r="AX5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AY5" s="157"/>
       <c r="AZ5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BA5" s="157"/>
       <c r="BB5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BC5" s="157"/>
       <c r="BD5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="BE5" s="157"/>
       <c r="BF5" s="182" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="BG5" s="157"/>
       <c r="BH5" s="156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="BI5" s="157"/>
       <c r="BJ5" s="156" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="BK5" s="157"/>
       <c r="BL5" s="156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="BM5" s="157"/>
       <c r="BN5" s="156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="BO5" s="157"/>
       <c r="BP5" s="156" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BQ5" s="157"/>
       <c r="BR5" s="156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="BS5" s="157"/>
     </row>
     <row r="6" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A6" s="14"/>
       <c r="B6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="F6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="H6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="J6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="L6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="N6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="P6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="R6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="T6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="U6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="U6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="V6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="X6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="Y6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Y6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="Z6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AA6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AA6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AB6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AC6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="AD6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AE6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AF6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AG6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AG6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AH6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AI6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AI6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AJ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AK6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AK6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AL6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AM6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AM6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AN6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AO6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AO6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AP6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AQ6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AQ6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="AR6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AS6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AS6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AT6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AU6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AU6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AV6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AW6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AW6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AX6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AY6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AY6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="AZ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BA6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BA6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BB6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BC6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BC6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BD6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BE6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="BE6" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="BF6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="BG6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BG6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BH6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BI6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BI6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BJ6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BK6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BK6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BL6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BM6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BM6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BN6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BO6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BO6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BP6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BQ6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BQ6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="BR6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="BS6" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="BS6" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -23926,7 +23923,7 @@
     </row>
     <row r="18" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A18" s="18" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="31"/>
@@ -24001,7 +23998,7 @@
     </row>
     <row r="19" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A19" s="82" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B19" s="79"/>
       <c r="C19" s="80"/>
@@ -24076,7 +24073,7 @@
     </row>
     <row r="20" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A20" s="82" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B20" s="32"/>
       <c r="C20" s="31"/>
@@ -24151,7 +24148,7 @@
     </row>
     <row r="21" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A21" s="82" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B21" s="32"/>
       <c r="C21" s="31"/>
@@ -24901,7 +24898,7 @@
     </row>
     <row r="31" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A31" s="18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B31" s="32"/>
       <c r="C31" s="31"/>
@@ -25049,7 +25046,7 @@
     </row>
     <row r="33" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A33" s="53" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B33" s="32"/>
       <c r="C33" s="31"/>
@@ -26584,7 +26581,7 @@
     </row>
     <row r="54" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A54" s="65" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B54" s="32"/>
       <c r="C54" s="31"/>
@@ -26659,7 +26656,7 @@
     </row>
     <row r="55" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A55" s="65" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B55" s="32"/>
       <c r="C55" s="31"/>
@@ -26734,7 +26731,7 @@
     </row>
     <row r="56" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A56" s="67" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B56" s="32"/>
       <c r="C56" s="31"/>
@@ -26745,7 +26742,7 @@
       <c r="H56" s="9"/>
       <c r="I56" s="10"/>
       <c r="J56" s="54" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K56" s="10"/>
       <c r="L56" s="33"/>
@@ -26811,7 +26808,7 @@
     </row>
     <row r="57" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A57" s="67" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B57" s="32"/>
       <c r="C57" s="31"/>
@@ -26842,7 +26839,7 @@
       <c r="AB57" s="33"/>
       <c r="AC57" s="35"/>
       <c r="AD57" s="49" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AE57" s="31"/>
       <c r="AF57" s="9"/>
@@ -26888,7 +26885,7 @@
     </row>
     <row r="58" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A58" s="67" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B58" s="32"/>
       <c r="C58" s="31"/>
@@ -26937,7 +26934,7 @@
       <c r="AT58" s="9"/>
       <c r="AU58" s="10"/>
       <c r="AV58" s="54" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AW58" s="10"/>
       <c r="AX58" s="9"/>
@@ -26965,7 +26962,7 @@
     </row>
     <row r="59" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A59" s="67" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B59" s="32"/>
       <c r="C59" s="31"/>
@@ -27332,7 +27329,7 @@
     </row>
     <row r="64" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A64" s="65" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B64" s="32"/>
       <c r="C64" s="31"/>
@@ -27407,7 +27404,7 @@
     </row>
     <row r="65" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A65" s="65" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B65" s="32"/>
       <c r="C65" s="31"/>
@@ -27482,10 +27479,10 @@
     </row>
     <row r="66" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A66" s="66" t="s">
+        <v>203</v>
+      </c>
+      <c r="B66" s="197" t="s">
         <v>204</v>
-      </c>
-      <c r="B66" s="197" t="s">
-        <v>205</v>
       </c>
       <c r="C66" s="198"/>
       <c r="D66" s="198"/>
@@ -27559,7 +27556,7 @@
     </row>
     <row r="67" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A67" s="66" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B67" s="165"/>
       <c r="C67" s="166"/>
@@ -27634,7 +27631,7 @@
     </row>
     <row r="68" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A68" s="66" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B68" s="165"/>
       <c r="C68" s="166"/>
@@ -27709,7 +27706,7 @@
     </row>
     <row r="69" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A69" s="66" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B69" s="201"/>
       <c r="C69" s="202"/>
@@ -27784,7 +27781,7 @@
     </row>
     <row r="70" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A70" s="66" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B70" s="32"/>
       <c r="C70" s="31"/>
@@ -27859,7 +27856,7 @@
     </row>
     <row r="71" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A71" s="66" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B71" s="32"/>
       <c r="C71" s="31"/>
@@ -27934,7 +27931,7 @@
     </row>
     <row r="72" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A72" s="66" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B72" s="32"/>
       <c r="C72" s="31"/>
@@ -28009,7 +28006,7 @@
     </row>
     <row r="73" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A73" s="66" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B73" s="32"/>
       <c r="C73" s="31"/>
@@ -28032,7 +28029,7 @@
       <c r="T73" s="9"/>
       <c r="U73" s="10"/>
       <c r="V73" s="196" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="W73" s="194"/>
       <c r="X73" s="194"/>
@@ -28042,7 +28039,7 @@
       <c r="AB73" s="33"/>
       <c r="AC73" s="35"/>
       <c r="AD73" s="193" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AE73" s="194"/>
       <c r="AF73" s="194"/>
@@ -28058,7 +28055,7 @@
       <c r="AP73" s="33"/>
       <c r="AQ73" s="35"/>
       <c r="AR73" s="79" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AS73" s="80"/>
       <c r="AT73" s="81"/>
@@ -28090,7 +28087,7 @@
     </row>
     <row r="74" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A74" s="66" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B74" s="32"/>
       <c r="C74" s="31"/>
@@ -28165,7 +28162,7 @@
     </row>
     <row r="75" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A75" s="66" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B75" s="32"/>
       <c r="C75" s="31"/>
@@ -28897,7 +28894,7 @@
     </row>
     <row r="85" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A85" s="18" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B85" s="32"/>
       <c r="C85" s="31"/>
@@ -28972,7 +28969,7 @@
     </row>
     <row r="86" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A86" s="15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B86" s="86"/>
       <c r="C86" s="87"/>
@@ -29047,7 +29044,7 @@
     </row>
     <row r="87" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A87" s="15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B87" s="32"/>
       <c r="C87" s="31"/>
@@ -29122,7 +29119,7 @@
     </row>
     <row r="88" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A88" s="45" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B88" s="32"/>
       <c r="C88" s="31"/>
@@ -29197,7 +29194,7 @@
     </row>
     <row r="89" spans="1:71" x14ac:dyDescent="0.2">
       <c r="A89" s="45" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B89" s="32"/>
       <c r="C89" s="31"/>
@@ -31024,7 +31021,7 @@
     </row>
     <row r="114" spans="1:71" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A114" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B114" s="176">
         <v>22</v>
@@ -31169,7 +31166,7 @@
     </row>
     <row r="115" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B115" s="153"/>
       <c r="C115" s="154"/>
@@ -31245,7 +31242,7 @@
     <row r="116" spans="1:71" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="177"/>
       <c r="B116" s="191" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C116" s="163"/>
       <c r="D116" s="163"/>
@@ -31261,7 +31258,7 @@
       <c r="N116" s="163"/>
       <c r="O116" s="164"/>
       <c r="P116" s="191" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="Q116" s="163"/>
       <c r="R116" s="163"/>
@@ -31277,7 +31274,7 @@
       <c r="AB116" s="163"/>
       <c r="AC116" s="164"/>
       <c r="AD116" s="191" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AE116" s="163"/>
       <c r="AF116" s="163"/>

</xml_diff>